<commit_message>
Refresh clinic_days and no_call_days with latest supervisor data
Both workbooks reloaded from the supervisor's current working copies.
All 67 tests pass and the full scheduler runs cleanly against the
updated inputs.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/clinic_days.xlsx
+++ b/data/clinic_days.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA2D4639-5D6D-4925-93A1-54255C0E2F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FC25A6C-E8C3-4ACE-AABA-C2AE2A7A1638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Block 1" sheetId="1" r:id="rId1"/>
@@ -1260,17 +1260,15 @@
         <v>46230</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F29" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
@@ -1324,7 +1322,7 @@
         <v>46232</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>6</v>
@@ -1389,11 +1387,9 @@
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K33" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
     <row r="34" spans="1:12">
@@ -4398,26 +4394,24 @@
         <v>46238</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -4434,7 +4428,9 @@
       <c r="C5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -4670,7 +4666,9 @@
       <c r="F14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -4778,7 +4776,9 @@
       <c r="H18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -4795,7 +4795,9 @@
       <c r="C19" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -4956,7 +4958,9 @@
       <c r="H25" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I25" s="2"/>
+      <c r="I25" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -5020,17 +5024,13 @@
         <v>9</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F28" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>28</v>
-      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>

</xml_diff>